<commit_message>
docs(product-d): add implementation action plan
</commit_message>
<xml_diff>
--- a/product-d/Riverside_Books_Product_D_Market_Research.xlsx
+++ b/product-d/Riverside_Books_Product_D_Market_Research.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Brief" sheetId="1" r:id="R13503f07a5dc4da0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Matrix" sheetId="2" r:id="R64b446e787bd444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Scorecard" sheetId="3" r:id="R71135860ea85472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Plan" sheetId="4" r:id="R5ff67eacaf94442f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R8c7c11cdbfd44c45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Brief" sheetId="1" r:id="Rfcd92d57b0514e1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Matrix" sheetId="2" r:id="Re2e0f59606794774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Scorecard" sheetId="3" r:id="Rd7f4872862504be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Plan" sheetId="4" r:id="Rb6398cd07f614287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R38ffa9775d724b85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="0.0"/>
+    <x:numFmt numFmtId="202" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -118,123 +119,43 @@
   <x:borders count="34">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="143">
+  <x:cellXfs count="144">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -564,6 +485,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -576,28 +500,28 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDEDED"/>
         </x:patternFill>
       </x:fill>
@@ -677,9 +601,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -744,7 +666,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R90020189fb074eb0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d96d7de2ef644e4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1394,7 +1316,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="96" t="str">
-        <x:v>Do NOT build a generic caption generator. Reuse CampaignFlow's proven interaction pattern, but redesign it around Riverside Books' shared schema. The MVP should make one task extremely easy: select a current book/event → generate several on-brand caption/post ideas → review/edit → copy or mark ready to publish.</x:v>
+        <x:v>Do NOT build a generic caption generator. Use a proven select → generate → review interaction pattern, redesigned around Riverside Books' shared schema. The MVP should make one task extremely easy: select a current book/event → generate several on-brand caption/post ideas → review/edit → copy or mark ready to publish.</x:v>
       </x:c>
       <x:c r="B34" s="78"/>
       <x:c r="C34" s="78"/>
@@ -2247,7 +2169,7 @@
       <x:c r="L4" s="26" t="str">
         <x:v>Buffer</x:v>
       </x:c>
-      <x:c r="M4" s="56" t="n">
+      <x:c r="M4" s="143" t="n">
         <x:f>I5</x:f>
         <x:v>84</x:v>
       </x:c>
@@ -2277,8 +2199,8 @@
       <x:c r="H5" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I5" s="56" t="n">
-        <x:f>(B5*$B$4+C5*$C$4+D5*$D$4+E5*$E$4+F5*$F$4+G5*$G$4+H5*$H$4)*20</x:f>
+      <x:c r="I5" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B5:H5)/SUM($B$4:$H$4)*20,0)</x:f>
         <x:v>84</x:v>
       </x:c>
       <x:c r="J5" s="26" t="str">
@@ -2287,9 +2209,9 @@
       <x:c r="L5" s="26" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="M5" s="56" t="n">
+      <x:c r="M5" s="143" t="n">
         <x:f>I6</x:f>
-        <x:v>69.99999999999999</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2317,9 +2239,9 @@
       <x:c r="H6" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="I6" s="56" t="n">
-        <x:f>(B6*$B$4+C6*$C$4+D6*$D$4+E6*$E$4+F6*$F$4+G6*$G$4+H6*$H$4)*20</x:f>
-        <x:v>69.99999999999999</x:v>
+      <x:c r="I6" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B6:H6)/SUM($B$4:$H$4)*20,0)</x:f>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="J6" s="26" t="str">
         <x:v>Good workflow; AI credits and limited data connection</x:v>
@@ -2327,9 +2249,9 @@
       <x:c r="L6" s="26" t="str">
         <x:v>Predis.ai</x:v>
       </x:c>
-      <x:c r="M6" s="56" t="n">
+      <x:c r="M6" s="143" t="n">
         <x:f>I7</x:f>
-        <x:v>84.99999999999999</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2357,9 +2279,9 @@
       <x:c r="H7" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I7" s="56" t="n">
-        <x:f>(B7*$B$4+C7*$C$4+D7*$D$4+E7*$E$4+F7*$F$4+G7*$G$4+H7*$H$4)*20</x:f>
-        <x:v>84.99999999999999</x:v>
+      <x:c r="I7" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B7:H7)/SUM($B$4:$H$4)*20,0)</x:f>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="J7" s="26" t="str">
         <x:v>Very strong creation; more complex than Riverside needs</x:v>
@@ -2367,9 +2289,9 @@
       <x:c r="L7" s="26" t="str">
         <x:v>Ocoya</x:v>
       </x:c>
-      <x:c r="M7" s="56" t="n">
+      <x:c r="M7" s="143" t="n">
         <x:f>I8</x:f>
-        <x:v>87.99999999999999</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -2397,9 +2319,9 @@
       <x:c r="H8" s="26" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I8" s="56" t="n">
-        <x:f>(B8*$B$4+C8*$C$4+D8*$D$4+E8*$E$4+F8*$F$4+G8*$G$4+H8*$H$4)*20</x:f>
-        <x:v>87.99999999999999</x:v>
+      <x:c r="I8" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B8:H8)/SUM($B$4:$H$4)*20,0)</x:f>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
         <x:v>Strongest data-to-content/automation analogue</x:v>
@@ -2407,7 +2329,7 @@
       <x:c r="L8" s="26" t="str">
         <x:v>SocialBee</x:v>
       </x:c>
-      <x:c r="M8" s="56" t="n">
+      <x:c r="M8" s="143" t="n">
         <x:f>I9</x:f>
         <x:v>79</x:v>
       </x:c>
@@ -2437,8 +2359,8 @@
       <x:c r="H9" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I9" s="56" t="n">
-        <x:f>(B9*$B$4+C9*$C$4+D9*$D$4+E9*$E$4+F9*$F$4+G9*$G$4+H9*$H$4)*20</x:f>
+      <x:c r="I9" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B9:H9)/SUM($B$4:$H$4)*20,0)</x:f>
         <x:v>79</x:v>
       </x:c>
       <x:c r="J9" s="26" t="str">
@@ -2447,7 +2369,7 @@
       <x:c r="L9" s="26" t="str">
         <x:v>Hootsuite</x:v>
       </x:c>
-      <x:c r="M9" s="56" t="n">
+      <x:c r="M9" s="143" t="n">
         <x:f>I10</x:f>
         <x:v>65</x:v>
       </x:c>
@@ -2477,8 +2399,8 @@
       <x:c r="H10" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I10" s="56" t="n">
-        <x:f>(B10*$B$4+C10*$C$4+D10*$D$4+E10*$E$4+F10*$F$4+G10*$G$4+H10*$H$4)*20</x:f>
+      <x:c r="I10" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B10:H10)/SUM($B$4:$H$4)*20,0)</x:f>
         <x:v>65</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
@@ -2487,7 +2409,7 @@
       <x:c r="L10" s="26" t="str">
         <x:v>Canva</x:v>
       </x:c>
-      <x:c r="M10" s="56" t="n">
+      <x:c r="M10" s="143" t="n">
         <x:f>I11</x:f>
         <x:v>80</x:v>
       </x:c>
@@ -2517,8 +2439,8 @@
       <x:c r="H11" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="I11" s="56" t="n">
-        <x:f>(B11*$B$4+C11*$C$4+D11*$D$4+E11*$E$4+F11*$F$4+G11*$G$4+H11*$H$4)*20</x:f>
+      <x:c r="I11" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B11:H11)/SUM($B$4:$H$4)*20,0)</x:f>
         <x:v>80</x:v>
       </x:c>
       <x:c r="J11" s="26" t="str">
@@ -2527,7 +2449,7 @@
       <x:c r="L11" s="26" t="str">
         <x:v>Adobe Express</x:v>
       </x:c>
-      <x:c r="M11" s="56" t="n">
+      <x:c r="M11" s="143" t="n">
         <x:f>I12</x:f>
         <x:v>82</x:v>
       </x:c>
@@ -2557,8 +2479,8 @@
       <x:c r="H12" s="26" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="I12" s="56" t="n">
-        <x:f>(B12*$B$4+C12*$C$4+D12*$D$4+E12*$E$4+F12*$F$4+G12*$G$4+H12*$H$4)*20</x:f>
+      <x:c r="I12" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B12:H12)/SUM($B$4:$H$4)*20,0)</x:f>
         <x:v>82</x:v>
       </x:c>
       <x:c r="J12" s="26" t="str">
@@ -2567,9 +2489,9 @@
       <x:c r="L12" s="26" t="str">
         <x:v>Jasper</x:v>
       </x:c>
-      <x:c r="M12" s="56" t="n">
+      <x:c r="M12" s="143" t="n">
         <x:f>I13</x:f>
-        <x:v>62.000000000000014</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -2597,9 +2519,9 @@
       <x:c r="H13" s="26" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I13" s="56" t="n">
-        <x:f>(B13*$B$4+C13*$C$4+D13*$D$4+E13*$E$4+F13*$F$4+G13*$G$4+H13*$H$4)*20</x:f>
-        <x:v>62.000000000000014</x:v>
+      <x:c r="I13" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B13:H13)/SUM($B$4:$H$4)*20,0)</x:f>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="J13" s="26" t="str">
         <x:v>Brand voice leader; no native social publishing</x:v>
@@ -2607,9 +2529,9 @@
       <x:c r="L13" s="26" t="str">
         <x:v>Copy.ai</x:v>
       </x:c>
-      <x:c r="M13" s="56" t="n">
+      <x:c r="M13" s="143" t="n">
         <x:f>I14</x:f>
-        <x:v>59.000000000000014</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -2637,9 +2559,9 @@
       <x:c r="H14" s="26" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I14" s="56" t="n">
-        <x:f>(B14*$B$4+C14*$C$4+D14*$D$4+E14*$E$4+F14*$F$4+G14*$G$4+H14*$H$4)*20</x:f>
-        <x:v>59.000000000000014</x:v>
+      <x:c r="I14" s="143" t="n">
+        <x:f>ROUND(SUMPRODUCT($B$4:$H$4,B14:H14)/SUM($B$4:$H$4)*20,0)</x:f>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="J14" s="26" t="str">
         <x:v>Strong workflow potential, weak social specialization</x:v>
@@ -2677,7 +2599,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R278db34b93364117"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf144bb1e1baf4201"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -2841,7 +2763,7 @@
         <x:v>Generate 3 variations.</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
-        <x:v>Gives staff choice and reuses a strong CampaignFlow interaction pattern.</x:v>
+        <x:v>Gives staff useful choice while keeping the select → generate → review pattern simple.</x:v>
       </x:c>
       <x:c r="E9" s="26" t="str">
         <x:v>Three distinct drafts appear from one selection.</x:v>
@@ -3282,7 +3204,9 @@
       <x:c r="E33" s="26" t="str">
         <x:v>Team 13</x:v>
       </x:c>
-      <x:c r="F33" s="122" t="str"/>
+      <x:c r="F33" s="122" t="str">
+        <x:v>Blocked — shared schema pending</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A34" s="93" t="str">
@@ -3300,9 +3224,11 @@
       <x:c r="E34" s="26" t="str">
         <x:v>Team 13</x:v>
       </x:c>
-      <x:c r="F34" s="122" t="str"/>
-    </x:row>
-    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="F34" s="122" t="str">
+        <x:v>Decided — Instagram + Facebook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A35" s="93" t="str">
         <x:v>Riverside brand voice</x:v>
       </x:c>
@@ -3318,7 +3244,9 @@
       <x:c r="E35" s="26" t="str">
         <x:v>Team 13</x:v>
       </x:c>
-      <x:c r="F35" s="122" t="str"/>
+      <x:c r="F35" s="122" t="str">
+        <x:v>Decided — warm, local, knowledgeable, community-focused</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A36" s="93" t="str">
@@ -3336,7 +3264,9 @@
       <x:c r="E36" s="26" t="str">
         <x:v>Crystal</x:v>
       </x:c>
-      <x:c r="F36" s="122" t="str"/>
+      <x:c r="F36" s="122" t="str">
+        <x:v>Decided — 3 variations</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A37" s="93" t="str">
@@ -3354,7 +3284,9 @@
       <x:c r="E37" s="26" t="str">
         <x:v>Team 13</x:v>
       </x:c>
-      <x:c r="F37" s="122" t="str"/>
+      <x:c r="F37" s="122" t="str">
+        <x:v>Decided — edit, copy, save draft, mark ready</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A38" s="93" t="str">
@@ -3372,7 +3304,9 @@
       <x:c r="E38" s="26" t="str">
         <x:v>Team 13</x:v>
       </x:c>
-      <x:c r="F38" s="122" t="str"/>
+      <x:c r="F38" s="122" t="str">
+        <x:v>Decided — text + post idea; visuals later</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A39" s="93" t="str">
@@ -3390,9 +3324,11 @@
       <x:c r="E39" s="26" t="str">
         <x:v>Ryan / Team</x:v>
       </x:c>
-      <x:c r="F39" s="122" t="str"/>
-    </x:row>
-    <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="F39" s="122" t="str">
+        <x:v>Product D decided — shared data; team contract pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A40" s="126" t="str">
         <x:v>Approval owner</x:v>
       </x:c>
@@ -3408,7 +3344,9 @@
       <x:c r="E40" s="127" t="str">
         <x:v>Team 13</x:v>
       </x:c>
-      <x:c r="F40" s="128" t="str"/>
+      <x:c r="F40" s="128" t="str">
+        <x:v>Decided — authenticated staff; no auto-publish</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>